<commit_message>
Update template and prevent duplicate
</commit_message>
<xml_diff>
--- a/public/Erection_Template.xlsx
+++ b/public/Erection_Template.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\00 Sources\sequencing\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01 Work\01 IBIM\01 Working\2026-04\sequencing\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4D4EDB6-1D05-4B0E-B4F6-12C757F928B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640"/>
   </bookViews>
   <sheets>
     <sheet name="#Erection_Stage_List" sheetId="2" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>ERECTION STAGE LIST</t>
   </si>
@@ -86,13 +85,16 @@
   </si>
   <si>
     <t>Assembly Name</t>
+  </si>
+  <si>
+    <t>{{PlanName}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="24" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="25">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -276,8 +278,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -466,6 +476,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -698,7 +714,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
@@ -736,6 +752,8 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1116,20 +1134,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" customWidth="1"/>
-    <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.625" customWidth="1"/>
+    <col min="2" max="2" width="16.625" customWidth="1"/>
+    <col min="3" max="3" width="16.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.875" customWidth="1"/>
+    <col min="6" max="6" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="37.15" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1140,22 +1158,22 @@
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
     </row>
-    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:7" ht="15" customHeight="1">
+      <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="14"/>
+      <c r="B3" s="16"/>
       <c r="C3" s="6"/>
       <c r="D3" s="7"/>
       <c r="E3" s="8"/>
       <c r="F3" s="9"/>
       <c r="G3" s="8"/>
     </row>
-    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+    <row r="4" spans="1:7" ht="15" customHeight="1">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="14"/>
+      <c r="B4" s="16"/>
       <c r="C4" s="6" t="s">
         <v>12</v>
       </c>
@@ -1164,33 +1182,33 @@
       <c r="F4" s="9"/>
       <c r="G4" s="8"/>
     </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
+    <row r="5" spans="1:7" ht="15" customHeight="1">
+      <c r="A5" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="14"/>
+      <c r="B5" s="16"/>
       <c r="C5" s="6"/>
       <c r="D5" s="7"/>
       <c r="E5" s="8"/>
       <c r="F5" s="9"/>
       <c r="G5" s="8"/>
     </row>
-    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+    <row r="6" spans="1:7" ht="15" customHeight="1">
+      <c r="A6" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="14"/>
+      <c r="B6" s="16"/>
       <c r="C6" s="6"/>
       <c r="D6" s="7"/>
       <c r="E6" s="8"/>
       <c r="F6" s="9"/>
       <c r="G6" s="8"/>
     </row>
-    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:7" ht="15" customHeight="1">
+      <c r="A7" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="14"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="6" t="s">
         <v>11</v>
       </c>
@@ -1199,7 +1217,7 @@
       <c r="F7" s="9"/>
       <c r="G7" s="8"/>
     </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="28.5">
       <c r="A10" s="10" t="s">
         <v>20</v>
       </c>
@@ -1222,34 +1240,41 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:7" ht="18.75" customHeight="1">
+      <c r="A12" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+    </row>
+    <row r="13" spans="1:7" ht="18.75" customHeight="1">
+      <c r="A13" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="F12" s="11"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="F13" s="11"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+    <row r="14" spans="1:7">
+      <c r="A14" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="F14" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="G13" s="2"/>
+      <c r="G14" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>